<commit_message>
feat(kepengasuhan): add dynamic excel export, interactive diff preview import, and guardian fields
</commit_message>
<xml_diff>
--- a/Setup_3_Santri_Wali_Putra_v2.xlsx
+++ b/Setup_3_Santri_Wali_Putra_v2.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ambisss\My Projek Laravel\elf_v1\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806F8F8E-8D23-4A1F-8B7E-2B82AA7FA1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Isian Data Santri" sheetId="1" r:id="rId4"/>
+    <sheet name="Isian Data Santri" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="999999"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="500">
   <si>
     <t>Nama Lengkap Santri *</t>
   </si>
@@ -1455,9 +1460,6 @@
   </si>
   <si>
     <t>Laju</t>
-  </si>
-  <si>
-    <t>Wali</t>
   </si>
   <si>
     <t>Naufal Riffat Mahanipuna</t>
@@ -1523,41 +1525,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="1"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color rgb="FF64748B"/>
       <name val="Calibri"/>
@@ -1638,26 +1627,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="5" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1947,32 +1944,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P132"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="true" style="0"/>
-    <col min="2" max="2" width="14" customWidth="true" style="0"/>
-    <col min="3" max="3" width="10" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12" customWidth="true" style="0"/>
-    <col min="5" max="5" width="18" customWidth="true" style="0"/>
-    <col min="6" max="6" width="18" customWidth="true" style="0"/>
-    <col min="7" max="7" width="10" customWidth="true" style="0"/>
-    <col min="8" max="8" width="28" customWidth="true" style="0"/>
-    <col min="9" max="9" width="15" customWidth="true" style="0"/>
-    <col min="10" max="10" width="20" customWidth="true" style="0"/>
-    <col min="11" max="11" width="28" customWidth="true" style="0"/>
-    <col min="12" max="12" width="18" customWidth="true" style="0"/>
-    <col min="13" max="13" width="15" customWidth="true" style="0"/>
-    <col min="14" max="14" width="35" customWidth="true" style="0"/>
-    <col min="15" max="15" width="35" customWidth="true" style="0"/>
-    <col min="16" max="16" width="14" customWidth="true" style="0"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="15" width="35" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" customHeight="1" ht="45">
+    <row r="1" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2022,7 +2014,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
@@ -2062,7 +2054,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>27</v>
       </c>
@@ -2104,7 +2096,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>31</v>
       </c>
@@ -2146,7 +2138,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>37</v>
       </c>
@@ -2188,7 +2180,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>43</v>
       </c>
@@ -2228,7 +2220,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>45</v>
       </c>
@@ -2270,7 +2262,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>51</v>
       </c>
@@ -2310,7 +2302,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
@@ -2352,7 +2344,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>58</v>
       </c>
@@ -2394,7 +2386,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>62</v>
       </c>
@@ -2436,7 +2428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>66</v>
       </c>
@@ -2478,7 +2470,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>71</v>
       </c>
@@ -2520,7 +2512,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>75</v>
       </c>
@@ -2562,7 +2554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>79</v>
       </c>
@@ -2604,7 +2596,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>84</v>
       </c>
@@ -2644,7 +2636,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>88</v>
       </c>
@@ -2684,7 +2676,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>92</v>
       </c>
@@ -2726,7 +2718,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>95</v>
       </c>
@@ -2766,7 +2758,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>97</v>
       </c>
@@ -2808,7 +2800,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>101</v>
       </c>
@@ -2850,7 +2842,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>105</v>
       </c>
@@ -2892,7 +2884,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>108</v>
       </c>
@@ -2934,7 +2926,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>113</v>
       </c>
@@ -2976,7 +2968,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>116</v>
       </c>
@@ -3018,7 +3010,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>121</v>
       </c>
@@ -3060,7 +3052,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>123</v>
       </c>
@@ -3102,7 +3094,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>128</v>
       </c>
@@ -3144,7 +3136,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>131</v>
       </c>
@@ -3186,7 +3178,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>135</v>
       </c>
@@ -3226,7 +3218,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>139</v>
       </c>
@@ -3266,7 +3258,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>141</v>
       </c>
@@ -3306,7 +3298,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>144</v>
       </c>
@@ -3346,7 +3338,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>146</v>
       </c>
@@ -3388,7 +3380,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>151</v>
       </c>
@@ -3430,7 +3422,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>155</v>
       </c>
@@ -3470,7 +3462,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>156</v>
       </c>
@@ -3512,7 +3504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>160</v>
       </c>
@@ -3554,7 +3546,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>167</v>
       </c>
@@ -3594,7 +3586,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>169</v>
       </c>
@@ -3636,7 +3628,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>173</v>
       </c>
@@ -3678,7 +3670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>177</v>
       </c>
@@ -3720,7 +3712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>181</v>
       </c>
@@ -3760,7 +3752,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>184</v>
       </c>
@@ -3802,7 +3794,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:16">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>188</v>
       </c>
@@ -3844,7 +3836,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>192</v>
       </c>
@@ -3886,7 +3878,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>196</v>
       </c>
@@ -3928,7 +3920,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>201</v>
       </c>
@@ -3970,7 +3962,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>206</v>
       </c>
@@ -4012,7 +4004,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>212</v>
       </c>
@@ -4054,7 +4046,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>216</v>
       </c>
@@ -4096,7 +4088,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>219</v>
       </c>
@@ -4138,7 +4130,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>223</v>
       </c>
@@ -4180,7 +4172,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>227</v>
       </c>
@@ -4220,7 +4212,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>231</v>
       </c>
@@ -4262,7 +4254,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>234</v>
       </c>
@@ -4304,7 +4296,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>239</v>
       </c>
@@ -4346,7 +4338,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:16">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>244</v>
       </c>
@@ -4388,7 +4380,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>247</v>
       </c>
@@ -4430,7 +4422,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>250</v>
       </c>
@@ -4472,7 +4464,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>253</v>
       </c>
@@ -4514,7 +4506,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:16">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>257</v>
       </c>
@@ -4556,7 +4548,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:16">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>261</v>
       </c>
@@ -4598,7 +4590,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:16">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>265</v>
       </c>
@@ -4640,7 +4632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:16">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>270</v>
       </c>
@@ -4682,7 +4674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:16">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>275</v>
       </c>
@@ -4724,7 +4716,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:16">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>280</v>
       </c>
@@ -4766,7 +4758,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:16">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>285</v>
       </c>
@@ -4808,7 +4800,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:16">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>289</v>
       </c>
@@ -4848,7 +4840,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:16">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>292</v>
       </c>
@@ -4890,7 +4882,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:16">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>295</v>
       </c>
@@ -4932,7 +4924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:16">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>299</v>
       </c>
@@ -4974,7 +4966,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:16">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>302</v>
       </c>
@@ -5016,7 +5008,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="74" spans="1:16">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>305</v>
       </c>
@@ -5058,7 +5050,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="75" spans="1:16">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>308</v>
       </c>
@@ -5098,7 +5090,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="76" spans="1:16">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>313</v>
       </c>
@@ -5140,7 +5132,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:16">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>319</v>
       </c>
@@ -5180,7 +5172,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:16">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>323</v>
       </c>
@@ -5222,7 +5214,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:16">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>328</v>
       </c>
@@ -5264,7 +5256,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:16">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>333</v>
       </c>
@@ -5306,7 +5298,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:16">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>338</v>
       </c>
@@ -5348,7 +5340,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:16">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>344</v>
       </c>
@@ -5390,7 +5382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:16">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>349</v>
       </c>
@@ -5432,7 +5424,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="84" spans="1:16">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>354</v>
       </c>
@@ -5474,7 +5466,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:16">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>359</v>
       </c>
@@ -5516,7 +5508,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:16">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>363</v>
       </c>
@@ -5558,7 +5550,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:16">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>367</v>
       </c>
@@ -5600,7 +5592,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:16">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>372</v>
       </c>
@@ -5640,7 +5632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:16">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>376</v>
       </c>
@@ -5680,7 +5672,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>380</v>
       </c>
@@ -5722,7 +5714,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>386</v>
       </c>
@@ -5764,7 +5756,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>390</v>
       </c>
@@ -5806,7 +5798,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>395</v>
       </c>
@@ -5848,7 +5840,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>399</v>
       </c>
@@ -5890,7 +5882,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>406</v>
       </c>
@@ -5932,7 +5924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:16">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>411</v>
       </c>
@@ -5974,7 +5966,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:16">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>416</v>
       </c>
@@ -6016,7 +6008,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:16">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>421</v>
       </c>
@@ -6058,7 +6050,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="99" spans="1:16">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>426</v>
       </c>
@@ -6100,7 +6092,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:16">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>431</v>
       </c>
@@ -6142,7 +6134,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:16">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>436</v>
       </c>
@@ -6184,7 +6176,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:16">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>439</v>
       </c>
@@ -6226,7 +6218,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:16">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>443</v>
       </c>
@@ -6268,7 +6260,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:16">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>448</v>
       </c>
@@ -6310,7 +6302,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:16">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>453</v>
       </c>
@@ -6352,7 +6344,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:16">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>457</v>
       </c>
@@ -6394,7 +6386,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:16">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>461</v>
       </c>
@@ -6436,7 +6428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:16">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>466</v>
       </c>
@@ -6478,7 +6470,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:16">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>471</v>
       </c>
@@ -6520,7 +6512,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:16">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>476</v>
       </c>
@@ -6562,7 +6554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:16">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
         <v>478</v>
       </c>
@@ -6581,24 +6573,16 @@
       <c r="J111" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K111" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L111" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M111" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K111" s="3"/>
+      <c r="L111" s="3"/>
+      <c r="M111" s="3"/>
       <c r="N111" s="3"/>
       <c r="O111" s="3"/>
-      <c r="P111" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="112" spans="1:16">
+      <c r="P111" s="3"/>
+    </row>
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -6615,24 +6599,16 @@
       <c r="J112" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K112" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L112" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M112" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K112" s="3"/>
+      <c r="L112" s="3"/>
+      <c r="M112" s="3"/>
       <c r="N112" s="3"/>
       <c r="O112" s="3"/>
-      <c r="P112" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="113" spans="1:16">
+      <c r="P112" s="3"/>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -6649,24 +6625,16 @@
       <c r="J113" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K113" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L113" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M113" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K113" s="3"/>
+      <c r="L113" s="3"/>
+      <c r="M113" s="3"/>
       <c r="N113" s="3"/>
       <c r="O113" s="3"/>
-      <c r="P113" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="114" spans="1:16">
+      <c r="P113" s="3"/>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -6683,24 +6651,16 @@
       <c r="J114" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K114" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L114" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M114" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K114" s="3"/>
+      <c r="L114" s="3"/>
+      <c r="M114" s="3"/>
       <c r="N114" s="3"/>
       <c r="O114" s="3"/>
-      <c r="P114" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="115" spans="1:16">
+      <c r="P114" s="3"/>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -6717,24 +6677,16 @@
       <c r="J115" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="K115" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L115" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M115" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K115" s="3"/>
+      <c r="L115" s="3"/>
+      <c r="M115" s="3"/>
       <c r="N115" s="3"/>
       <c r="O115" s="3"/>
-      <c r="P115" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="116" spans="1:16">
+      <c r="P115" s="3"/>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -6751,24 +6703,16 @@
       <c r="J116" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="K116" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L116" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M116" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K116" s="3"/>
+      <c r="L116" s="3"/>
+      <c r="M116" s="3"/>
       <c r="N116" s="3"/>
       <c r="O116" s="3"/>
-      <c r="P116" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="117" spans="1:16">
+      <c r="P116" s="3"/>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -6785,24 +6729,16 @@
       <c r="J117" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="K117" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L117" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M117" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K117" s="3"/>
+      <c r="L117" s="3"/>
+      <c r="M117" s="3"/>
       <c r="N117" s="3"/>
       <c r="O117" s="3"/>
-      <c r="P117" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="118" spans="1:16">
+      <c r="P117" s="3"/>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -6819,24 +6755,16 @@
       <c r="J118" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K118" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L118" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M118" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K118" s="3"/>
+      <c r="L118" s="3"/>
+      <c r="M118" s="3"/>
       <c r="N118" s="3"/>
       <c r="O118" s="3"/>
-      <c r="P118" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="119" spans="1:16">
+      <c r="P118" s="3"/>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -6853,24 +6781,16 @@
       <c r="J119" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K119" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L119" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M119" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K119" s="3"/>
+      <c r="L119" s="3"/>
+      <c r="M119" s="3"/>
       <c r="N119" s="3"/>
       <c r="O119" s="3"/>
-      <c r="P119" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="120" spans="1:16">
+      <c r="P119" s="3"/>
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -6887,24 +6807,16 @@
       <c r="J120" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K120" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L120" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M120" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K120" s="3"/>
+      <c r="L120" s="3"/>
+      <c r="M120" s="3"/>
       <c r="N120" s="3"/>
       <c r="O120" s="3"/>
-      <c r="P120" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="121" spans="1:16">
+      <c r="P120" s="3"/>
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -6921,24 +6833,16 @@
       <c r="J121" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K121" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L121" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M121" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K121" s="3"/>
+      <c r="L121" s="3"/>
+      <c r="M121" s="3"/>
       <c r="N121" s="3"/>
       <c r="O121" s="3"/>
-      <c r="P121" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="122" spans="1:16">
+      <c r="P121" s="3"/>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -6955,24 +6859,16 @@
       <c r="J122" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K122" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L122" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M122" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K122" s="3"/>
+      <c r="L122" s="3"/>
+      <c r="M122" s="3"/>
       <c r="N122" s="3"/>
       <c r="O122" s="3"/>
-      <c r="P122" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="123" spans="1:16">
+      <c r="P122" s="3"/>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -6989,24 +6885,16 @@
       <c r="J123" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K123" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L123" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M123" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K123" s="3"/>
+      <c r="L123" s="3"/>
+      <c r="M123" s="3"/>
       <c r="N123" s="3"/>
       <c r="O123" s="3"/>
-      <c r="P123" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="124" spans="1:16">
+      <c r="P123" s="3"/>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -7023,24 +6911,16 @@
       <c r="J124" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K124" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L124" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M124" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K124" s="3"/>
+      <c r="L124" s="3"/>
+      <c r="M124" s="3"/>
       <c r="N124" s="3"/>
       <c r="O124" s="3"/>
-      <c r="P124" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="125" spans="1:16">
+      <c r="P124" s="3"/>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -7057,24 +6937,16 @@
       <c r="J125" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K125" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L125" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M125" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K125" s="3"/>
+      <c r="L125" s="3"/>
+      <c r="M125" s="3"/>
       <c r="N125" s="3"/>
       <c r="O125" s="3"/>
-      <c r="P125" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="126" spans="1:16">
+      <c r="P125" s="3"/>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -7091,24 +6963,16 @@
       <c r="J126" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K126" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L126" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M126" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K126" s="3"/>
+      <c r="L126" s="3"/>
+      <c r="M126" s="3"/>
       <c r="N126" s="3"/>
       <c r="O126" s="3"/>
-      <c r="P126" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="127" spans="1:16">
+      <c r="P126" s="3"/>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -7125,24 +6989,16 @@
       <c r="J127" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K127" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L127" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M127" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K127" s="3"/>
+      <c r="L127" s="3"/>
+      <c r="M127" s="3"/>
       <c r="N127" s="3"/>
       <c r="O127" s="3"/>
-      <c r="P127" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="128" spans="1:16">
+      <c r="P127" s="3"/>
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -7159,24 +7015,16 @@
       <c r="J128" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K128" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L128" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M128" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K128" s="3"/>
+      <c r="L128" s="3"/>
+      <c r="M128" s="3"/>
       <c r="N128" s="3"/>
       <c r="O128" s="3"/>
-      <c r="P128" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="129" spans="1:16">
+      <c r="P128" s="3"/>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -7193,24 +7041,16 @@
       <c r="J129" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K129" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L129" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M129" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K129" s="3"/>
+      <c r="L129" s="3"/>
+      <c r="M129" s="3"/>
       <c r="N129" s="3"/>
       <c r="O129" s="3"/>
-      <c r="P129" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="130" spans="1:16">
+      <c r="P129" s="3"/>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -7227,38 +7067,19 @@
       <c r="J130" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K130" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L130" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="M130" s="3" t="s">
-        <v>480</v>
-      </c>
+      <c r="K130" s="3"/>
+      <c r="L130" s="3"/>
+      <c r="M130" s="3"/>
       <c r="N130" s="3"/>
       <c r="O130" s="3"/>
-      <c r="P130" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="132" spans="1:16">
+      <c r="P130" s="3"/>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>